<commit_message>
Revise Q3 prioritization: remove done/cancelled items, fix 4W readiness
- X-dock: remove "Adjust No. Invoice standardization" (already done); renumber.
- Scheduled Instant: remove "NCS API integration" (cancelled) and remove
  "Phase 2 automated WA confirm loop" + "Calendar Schedule Metrics" (already
  done); merge "Standardize bulk-upload template" + "AI CSV header-checker"
  into one item (template committed, AI a feasibility spike — two paths to one
  problem); renumber.
- 4W: correct readiness on all items to "needs PRD/prototype" — the recap
  next-steps are not yet built, so September is scope-and-build. Cover +
  subtitle note this; September-commitment confidence updated accordingly.
- Add Rev 2 change-log row to the Cover tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PKPvRHH13fns55VRTHV1kP
</commit_message>
<xml_diff>
--- a/docs/prioritization/q3-2026-prioritization-v1.xlsx
+++ b/docs/prioritization/q3-2026-prioritization-v1.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Signals how fast an item can move. 'Prototype + PRD' = buildable now · 'Prototype only' / 'PRD only' = one artifact missing · 'Draft' = early · 'None — needs PRD' = requirement gathering first · 'Spike / feasibility' = go/no-go pending. Readiness is why some P0s still land later than P1 quick-wins.</t>
+          <t>Signals how fast an item can move. 'Prototype + PRD' = buildable now · 'Prototype only' / 'PRD only' = one artifact missing · 'Draft' = early · 'None — needs PRD/prototype' = requirement gathering first · 'Spike / feasibility' = go/no-go pending. IMPORTANT: every 4W September item still needs PRD + prototype — September for 4W means scope-and-build, so write those PRDs in the first days of the month; the P0s are small (≈1pw each) so this is achievable but not free.</t>
         </is>
       </c>
     </row>
@@ -732,123 +732,135 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Rev 2 (31 Aug)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Removed as already done: X-dock 'Adjust No. Invoice standardization'; SI 'Phase 2 automated WA confirm loop' and 'Calendar Schedule Metrics'. Removed as cancelled: SI 'NCS API integration'. Merged into one item: SI 'Standardize bulk-upload template' + 'AI CSV header-checker' (two paths to one problem — template committed, AI a feasibility spike). Corrected: all 4W items marked 'needs PRD/prototype' (the recap next-steps are not yet built).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Priority swatches</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Must-ship this cycle</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Important, schedulable</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Nice-to-have / deferred</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Month swatches</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Committed September slate</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Next — October</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Later / large-scope / blocked</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Awaiting business decision</t>
         </is>
@@ -869,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -951,7 +963,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Adjust No. Invoice (TMP-INV) standardization</t>
+          <t>COD Phase 1 — reconciliation</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -961,7 +973,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>In progress (PRD ✓)</t>
+          <t>Prototype + PRD ✓</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -993,7 +1005,7 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>COD Phase 1 — reconciliation</t>
+          <t>Retry Shipment</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1003,7 +1015,7 @@
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -1011,14 +1023,14 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Buku Warung onboarding</t>
         </is>
       </c>
     </row>
@@ -1035,17 +1047,17 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Retry Shipment</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>None — needs PRD</t>
+          <t>Prototype + PRD ✓</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1053,41 +1065,41 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Buku Warung onboarding</t>
+          <t>Mobile engineer slot</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>X-dock</t>
+          <t>Scheduled Instant</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>XD-04</t>
+          <t>SI-01</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Exception blast WhatsApp — Noovoleum</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>Spike</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
@@ -1095,14 +1107,14 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H8" s="19" t="inlineStr">
         <is>
-          <t>Mobile engineer slot</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1114,12 +1126,12 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>SI-01</t>
+          <t>SI-02</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Integrasi API &amp; sistem shipment request — NCS</t>
+          <t>Pricing per shift</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1129,7 +1141,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Preparation (PRD in progress)</t>
+          <t>Prototype + PRD ✓ (pending business)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1144,24 +1156,24 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Business pricing decision</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>Scheduled Instant</t>
+          <t>4W</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>SI-02</t>
+          <t>NS-DA-01</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Exception blast WhatsApp — Noovoleum</t>
+          <t>Move completed shipment from Beranda → Riwayat</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1171,7 +1183,7 @@
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Spike</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
@@ -1193,17 +1205,17 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>Scheduled Instant</t>
+          <t>4W</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>SI-03</t>
+          <t>NS-MTH-01</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Pricing per shift</t>
+          <t>Cancel Shipment (human-error from UJP)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1213,7 +1225,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓ (pending business)</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1228,34 +1240,34 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Business pricing decision</t>
+          <t>UJP bridge (import-only)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Scheduled Instant</t>
+          <t>4W</t>
         </is>
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>SI-04</t>
+          <t>NS-MTH-02</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>SI Phase 2 — automated WhatsApp confirmation loop (T-12 / T-2)</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Mark as Completed / Mark as Failed (Ops override)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>PRD (Phase 2 defined)</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="F12" s="19" t="inlineStr">
@@ -1263,9 +1275,9 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H12" s="19" t="inlineStr">
@@ -1282,22 +1294,22 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>NS-DA-01</t>
+          <t>NS-DL-01</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Move completed shipment from Beranda → Riwayat</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>EXIM Import/Export tagging (consumer)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1305,14 +1317,14 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NS-MTH-03 (Mithril tag)</t>
         </is>
       </c>
     </row>
@@ -1324,22 +1336,22 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>NS-MTH-01</t>
+          <t>NS-MTH-03</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>Cancel Shipment (human-error from UJP)</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>EXIM Import/Export tagging</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
@@ -1347,14 +1359,14 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>UJP bridge (import-only)</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1366,22 +1378,22 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>NS-MTH-02</t>
+          <t>NS-DA-03</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Mark as Completed / Mark as Failed (Ops override)</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>Push Notifications (full set — see Tab 6)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD (Wave 1)</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1389,138 +1401,12 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>NS-DL-01</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>EXIM Import/Export tagging (consumer)</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>Depends on NS-MTH-03</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>NS-MTH-03</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>EXIM Import/Export tagging</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Prototype + PRD ✓</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>NS-DA-03</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Push Notifications (full set — see Tab 6)</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>PRD ✓ (Wave 1)</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>NS-MTH-01, NS-MTH-02</t>
         </is>
@@ -1572,7 +1458,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap; Target-month phasing + readiness added.</t>
+          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap; Target-month phasing + readiness added. Note: all September items still need PRD/prototype — September is scope-and-build.</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1598,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -1785,7 +1671,7 @@
       </c>
       <c r="L6" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="M6" s="19" t="inlineStr">
@@ -1858,7 +1744,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -1931,7 +1817,7 @@
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Depends on NS-MTH-03</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
@@ -2004,7 +1890,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -2077,7 +1963,7 @@
       </c>
       <c r="L10" s="19" t="inlineStr">
         <is>
-          <t>PRD ✓ (Wave 1)</t>
+          <t>None — needs PRD (Wave 1)</t>
         </is>
       </c>
       <c r="M10" s="19" t="inlineStr">
@@ -2296,7 +2182,7 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Depends on NS-MTH-03</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -2627,7 +2513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2658,7 +2544,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scheduled Instant — rider scheduling &amp; shipment intake. September = NCS API prep, Noovoleum WA exception, pricing per shift, SI Phase 2 confirm loop.</t>
+          <t>Scheduled Instant — rider scheduling &amp; shipment intake. September = Noovoleum WA exception + pricing per shift. Removed: NCS API integration (cancelled), Phase 2 WA confirm loop &amp; Calendar metrics (already done).</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2638,7 @@
     <row r="5" ht="118" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>SI-03</t>
+          <t>SI-02</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -2830,30 +2716,30 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Integration</t>
+          <t>WA / Backend</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Integrasi API &amp; sistem shipment request — NCS</t>
+          <t>Exception blast WhatsApp — Noovoleum</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ingest shipment requests from client NCS automatically via API, so orders no longer have to be keyed in by hand.</t>
+          <t>Client-specific exception to the WhatsApp blast rules for Noovoleum riders.</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I6" s="25">
         <f>(E6*F6*G6)/H6</f>
@@ -2871,7 +2757,7 @@
       </c>
       <c r="L6" s="19" t="inlineStr">
         <is>
-          <t>Preparation (PRD in progress)</t>
+          <t>Spike</t>
         </is>
       </c>
       <c r="M6" s="19" t="inlineStr">
@@ -2891,39 +2777,39 @@
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>Unblocks NCS scale and removes manual order entry — the biggest Ops-friction reducer in the SI backlog. Preparation is underway; integration itself runs ~1 month, so it starts in September even if it finishes early October.</t>
+          <t>Client commitment, currently being spiked by engineering. Small in scope but client-blocking, so it rides with the September P0 slate.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>SI-02</t>
+          <t>SI-03</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>WA / Backend</t>
+          <t>Mithril / Schedule</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Exception blast WhatsApp — Noovoleum</t>
+          <t>Filter cari per rider (POV rider)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Client-specific exception to the WhatsApp blast rules for Noovoleum riders.</t>
+          <t>See every client a single rider is assigned to on a given day (this view lives today in an Ops-built internal tool).</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="H7" s="20" t="n">
         <v>1</v>
@@ -2932,19 +2818,19 @@
         <f>(E7*F7*G7)/H7</f>
         <v/>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>Sep</t>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Spike</t>
+          <t>PRD only</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -2964,7 +2850,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>Client commitment, currently being spiked by engineering. Small in scope but client-blocking, so it rides with the September P0 slate.</t>
+          <t>Replaces a manual Ops workaround with a native view. Useful but not launch-blocking → October.</t>
         </is>
       </c>
     </row>
@@ -2976,30 +2862,30 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>WA / Backend</t>
+          <t>Web / Back Office (+AI spike)</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>SI Phase 2 — automated WhatsApp confirmation loop (T-12 / T-2)</t>
+          <t>Standardize bulk-upload template + AI header-checker (feasibility)</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Automated confirmation pings at T-12h and T-2h to lift rider response rate (today 'No Response' dominates the confirmation funnel).</t>
+          <t>One initiative, two paths to the same goal — let clients self-upload orders without the Ops team, cutting human error. Path A (committed): standardize the bulk-upload template header so uploads are consistent across clients. Path B (spike): an AI that auto-validates arbitrary/dynamic client CSV headers.</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" s="23" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I8" s="25">
         <f>(E8*F8*G8)/H8</f>
@@ -3010,14 +2896,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>Sep</t>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
         </is>
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>PRD (Phase 2 defined)</t>
+          <t>Draft template (AI = feasibility spike)</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
@@ -3032,12 +2918,12 @@
       </c>
       <c r="O8" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Speaker 1 CSV analysis</t>
         </is>
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Directly targets the gap the live feature exposed: adoption/coverage is up but confirmation is still weak. Pairs with Ops socialization + the Rp5.000 no-response deduction. High reach (every slot). P1 by tier but sequenced into late September because it's the highest-leverage follow-through on a shipped feature.</t>
+          <t>These are two solutions to one problem, so they're tracked as one item. A draft template already exists (Path A). The meeting explored the AI header-checker (Path B) but engineering judged the effort very large — client templates are highly dynamic, manual validation is still needed up front, and pulling supporting data (e.g. customer records) is hard. Decision: commit to standardizing the template first; run the AI checker only as a time-boxed feasibility spike whose go/no-go rests on Speaker 1's analysis of NCS's sample CSV. If the AI path isn't feasible, we keep the standardized template and drop the AI work. Confidence held at 0.55 because the committed scope (template) is clear but the AI upside is unproven.</t>
         </is>
       </c>
     </row>
@@ -3049,48 +2935,48 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Schedule</t>
+          <t>TBC</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Calendar — Schedule Metrics</t>
+          <t>Sayurbox — Tender Sistem</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Render performance metrics directly inside the Schedule calendar.</t>
+          <t>System tender for Sayurbox.</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I9" s="22">
         <f>(E9*F9*G9)/H9</f>
         <v/>
       </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>TBC</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Prototype ready</t>
+          <t>TBC — business / leads</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -3105,302 +2991,10 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Business &amp; Leads scope</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>Prototype ready. Ops-visibility polish rather than a blocker — October, once the P0 integration work is moving.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="118" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>SI-07</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Web / Back Office</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Standardize bulk-upload template header</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Standardize the shipment bulk-upload template header so uploads are consistent across clients (whose formats differ today) and need less Ops hand-holding.</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="24" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H10" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" s="25">
-        <f>(E10*F10*G10)/H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L10" s="19" t="inlineStr">
-        <is>
-          <t>Draft template only</t>
-        </is>
-      </c>
-      <c r="M10" s="19" t="inlineStr">
-        <is>
-          <t>Isumi Karina</t>
-        </is>
-      </c>
-      <c r="N10" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="O10" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P10" s="19" t="inlineStr">
-        <is>
-          <t>A draft template already exists. The meeting explored an AI header-checker to auto-validate uploads, but engineering judged the effort very large (client templates are highly dynamic, manual validation is still needed up front, and pulling supporting data e.g. customer records is hard). Decision: standardize the template first; treat AI checking as a separate feasibility spike (SI-08). Confidence held at 0.60 until the template logic is proven on a real client sample.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="118" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>SI-06</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Mithril / Schedule</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Filter cari per rider (POV rider)</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>See every client a single rider is assigned to on a given day (this view lives today in an Ops-built internal tool).</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="21" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="22">
-        <f>(E11*F11*G11)/H11</f>
-        <v/>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>PRD only</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>Isumi Karina</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P11" s="4" t="inlineStr">
-        <is>
-          <t>Replaces a manual Ops workaround with a native view. Useful but not launch-blocking → October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="118" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>SI-08</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Web / Backend / AI</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>AI CSV header-checker (feasibility spike)</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>AI that auto-validates client CSV headers so clients can self-upload orders without the Ops team, cutting human error.</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="H12" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="I12" s="25">
-        <f>(E12*F12*G12)/H12</f>
-        <v/>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="L12" s="19" t="inlineStr">
-        <is>
-          <t>Spike — feasibility TBD</t>
-        </is>
-      </c>
-      <c r="M12" s="19" t="inlineStr">
-        <is>
-          <t>Isumi Karina</t>
-        </is>
-      </c>
-      <c r="N12" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="O12" s="19" t="inlineStr">
-        <is>
-          <t>Speaker 1 CSV analysis, SI-07</t>
-        </is>
-      </c>
-      <c r="P12" s="19" t="inlineStr">
-        <is>
-          <t>The meeting flagged this as high-effort, low-certainty. Go/no-go rests on Speaker 1's analysis of NCS's sample CSV template and logic — if it isn't feasible, the project stops and we lean on SI-07 instead. Keep it a time-boxed spike, not a committed build; that's why confidence is 0.35.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="118" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>SI-09</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Sayurbox — Tender Sistem</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>System tender for Sayurbox.</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="I13" s="22">
-        <f>(E13*F13*G13)/H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>TBC — business / leads</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>Isumi Karina</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>Business &amp; Leads scope</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Detail and context are incomplete — still TBC with Business &amp; Leads. Cannot be scoped or scheduled until they define the requirement, so it sits outside the month plan for now.</t>
         </is>
@@ -3421,7 +3015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3452,7 +3046,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-docking — goal: move all cross-dock clients to the new app. September = invoice-no. standardization, COD Phase 1, retry shipment, scan-doc/leave-at-outlet.</t>
+          <t>Cross-docking — goal: move all cross-dock clients to the new app. September = COD Phase 1, retry shipment, scan-doc/leave-at-outlet. Removed: Adjust No. Invoice standardization (already done).</t>
         </is>
       </c>
     </row>
@@ -3546,22 +3140,22 @@
     <row r="5" ht="118" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>XD-01</t>
+          <t>XD-02</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Web+Mobile</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Adjust No. Invoice (TMP-INV) standardization</t>
+          <t>Retry Shipment</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Standardize the new invoice no. TMP-INV-XXX across every X-dock flow: import shipment, POD per package (shown in mobile), scan inbound &amp; driver batch scan, AI Checker, pending invoices, and back-office bulk upload (Invoice + Koli columns). SwipeRX: Invoice column mandatory.</t>
+          <t>Auto-retry failed deliveries (e.g. pharmacy closed) with a structured re-attempt instead of manual re-create. Needed across many clients — Buku Warung and SwipeRX called out.</t>
         </is>
       </c>
       <c r="E5" s="20" t="n">
@@ -3571,10 +3165,10 @@
         <v>3</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="H5" s="20" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I5" s="22">
         <f>(E5*F5*G5)/H5</f>
@@ -3592,7 +3186,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>In progress (PRD ✓)</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -3607,47 +3201,47 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Buku Warung onboarding</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Core cross-docking hardening the 28-Aug meeting called out ('perfect cross-docking'). One consistent invoice number is the backbone for clean invoice tracking across all X-dock clients — already in dev, so it lands in September.</t>
+          <t>Top of the meeting's priority list and highest reach (multi-client). But no PRD or prototype yet, so confidence is held at 0.70: run requirement gathering in the first week of September, then build. Buku Warung targets go-live W2–W3 September with API integration accepted as not-ready-at-launch (~1 month grace) — retry is what keeps that onboarding reliable, so it stays a September P0 even though the build may finish end-of-month.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="118" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>XD-03</t>
+          <t>XD-01</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Driver App</t>
+          <t>Mithril / Back Office</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Retry Shipment</t>
+          <t>COD Phase 1 — reconciliation</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Auto-retry failed deliveries (e.g. pharmacy closed) with a structured re-attempt instead of manual re-create. Needed across many clients — Buku Warung and SwipeRX called out.</t>
+          <t>Record and reconcile Cash-on-Delivery collected per shipment (Zalora). Scope is reconciliation only — no payment-gateway link yet.</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I6" s="25">
         <f>(E6*F6*G6)/H6</f>
@@ -3665,7 +3259,7 @@
       </c>
       <c r="L6" s="19" t="inlineStr">
         <is>
-          <t>None — needs PRD</t>
+          <t>Prototype + PRD ✓</t>
         </is>
       </c>
       <c r="M6" s="19" t="inlineStr">
@@ -3680,44 +3274,44 @@
       </c>
       <c r="O6" s="19" t="inlineStr">
         <is>
-          <t>Buku Warung onboarding</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>Top of the meeting's priority list and highest reach (multi-client). But no PRD or prototype yet, so confidence is held at 0.70: run requirement gathering in the first week of September, then build. Buku Warung targets go-live W2–W3 September with API integration accepted as not-ready-at-launch (~1 month grace) — retry is what keeps that onboarding reliable, so it stays a September P0 even though the build may finish end-of-month.</t>
+          <t>Active focus per the meeting: one engineer paused 'upload performance' to concentrate on COD, working to Albert's PRD. Prototype + PRD are ready and scope is deliberately narrow (reconciliation), so it fits September. Phase 2 (payment-gateway QRIS auto-check) is split out as XD-07.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>XD-02</t>
+          <t>XD-03</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Back Office</t>
+          <t>Driver App (Mobile)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>COD Phase 1 — reconciliation</t>
+          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Record and reconcile Cash-on-Delivery collected per shipment (Zalora). Scope is reconciliation only — no payment-gateway link yet.</t>
+          <t>Driver handles multiple invoices in one outlet visit, plus a 'leave at outlet' option with a scanned blank-document (BAST) as proof.</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="H7" s="20" t="n">
         <v>1.5</v>
@@ -3726,9 +3320,9 @@
         <f>(E7*F7*G7)/H7</f>
         <v/>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
@@ -3753,12 +3347,12 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mobile engineer slot</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>Active focus per the meeting: one engineer paused 'upload performance' to concentrate on COD, working to Albert's PRD. Prototype + PRD are ready and scope is deliberately narrow (reconciliation), so it fits September. Phase 2 (payment-gateway QRIS auto-check) is split out as XD-08.</t>
+          <t>Prototype + PRD ready and a mobile engineer is confirmed to pick it up Thursday 3 September — a clean September win. Cuts failed-visit re-dispatch and matches how drivers actually work outlets.</t>
         </is>
       </c>
     </row>
@@ -3770,27 +3364,27 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Driver App (Mobile)</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
+          <t>Shipment Bypass Hub — SwipeRX</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Driver handles multiple invoices in one outlet visit, plus a 'leave at outlet' option with a scanned blank-document (BAST) as proof.</t>
+          <t>Rider rides the van from the Tempe warehouse straight to the pharmacy, bypassing the Dash hub. Uses Create Shipment with origin = client hub.</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" s="23" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H8" s="23" t="n">
         <v>1.5</v>
@@ -3804,14 +3398,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>Sep</t>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
         </is>
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓</t>
+          <t>Prototype ready</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
@@ -3826,47 +3420,47 @@
       </c>
       <c r="O8" s="19" t="inlineStr">
         <is>
-          <t>Mobile engineer slot</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Prototype + PRD ready and a mobile engineer is confirmed to pick it up Thursday 3 September — a clean September win. Cuts failed-visit re-dispatch and matches how drivers actually work outlets.</t>
+          <t>Prototype is ready, status pending. SwipeRX-specific and not blocking any September launch, so schedule right after the P0 cluster in October.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="118" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>XD-06</t>
+          <t>XD-05</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Driver App</t>
+          <t>Mithril</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Shipment Bypass Hub — SwipeRX</t>
+          <t>Filter client X-dock in Schedule menu</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Rider rides the van from the Tempe warehouse straight to the pharmacy, bypassing the Dash hub. Uses Create Shipment with origin = client hub.</t>
+          <t>X-dock shares the Schedule calendar (default filter is currently Scheduled Instant); it needs a per-squad filter. The X-dock calendar stays empty until requirement gathering fills it.</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I9" s="22">
         <f>(E9*F9*G9)/H9</f>
@@ -3884,7 +3478,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Prototype ready</t>
+          <t>PRD partial — needs detail</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -3904,29 +3498,29 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Prototype is ready, status pending. SwipeRX-specific and not blocking any September launch, so schedule right after the P0 cluster in October.</t>
+          <t>Detail depends on requirement gathering that hasn't happened; low urgency next to the P0 cluster, so October. The filter itself is small — the calendar content behind it is the real open question.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="118" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>XD-05</t>
+          <t>XD-06</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Mithril</t>
+          <t>Mithril / Dash Link</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Filter client X-dock in Schedule menu</t>
+          <t>Performance invoice — POV outlet</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>X-dock shares the Schedule calendar (default filter is currently Scheduled Instant); it needs a per-squad filter. The X-dock calendar stays empty until requirement gathering fills it.</t>
+          <t>Invoice performance from the outlet's point of view (Logistic Mithril &amp; Dash Link). Primarily a client request.</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
@@ -3936,7 +3530,7 @@
         <v>1</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="H10" s="23" t="n">
         <v>1</v>
@@ -3945,9 +3539,9 @@
         <f>(E10*F10*G10)/H10</f>
         <v/>
       </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -3957,7 +3551,7 @@
       </c>
       <c r="L10" s="19" t="inlineStr">
         <is>
-          <t>PRD partial — needs detail</t>
+          <t>Prototype + PRD ✓ (paused)</t>
         </is>
       </c>
       <c r="M10" s="19" t="inlineStr">
@@ -3977,7 +3571,7 @@
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>Detail depends on requirement gathering that hasn't happened; low urgency next to the P0 cluster, so October. The filter itself is small — the calendar content behind it is the real open question.</t>
+          <t>Ready but deliberately paused: per the meeting, the engineer moved off 'upload performance' onto COD. Resume in October once COD Phase 1 is stable. Low reach (reporting view), so P2 despite being buildable.</t>
         </is>
       </c>
     </row>
@@ -3989,30 +3583,30 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Dash Link</t>
+          <t>Mithril / Back Office + PG</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Performance invoice — POV outlet</t>
+          <t>COD Phase 2 — Payment Gateway QRIS auto-check</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Invoice performance from the outlet's point of view (Logistic Mithril &amp; Dash Link). Primarily a client request.</t>
+          <t>Connect COD to the Payment Gateway to auto-verify QRIS payment, replacing Phase 1's manual reconciliation.</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="21" t="n">
-        <v>0.85</v>
+        <v>0.6</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11" s="22">
         <f>(E11*F11*G11)/H11</f>
@@ -4023,14 +3617,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ✓ (paused)</t>
+          <t>None — needs PRD</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -4045,12 +3639,12 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>XD-01 (Phase 1), PG integration</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Ready but deliberately paused: per the meeting, the engineer moved off 'upload performance' onto COD. Resume in October once COD Phase 1 is stable. Low reach (reporting view), so P2 despite being buildable.</t>
+          <t>Builds on Phase 1. External payment-gateway dependency plus no PRD yet → confidence low and effort high, so Q4. Sequencing: only start once Phase 1 reconciliation is live and the PG contract/scope is settled.</t>
         </is>
       </c>
     </row>
@@ -4062,43 +3656,43 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Back Office + PG</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>COD Phase 2 — Payment Gateway QRIS auto-check</t>
+          <t>Dispatch &amp; Pick-up (drop + pickup in one trip)</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Connect COD to the Payment Gateway to auto-verify QRIS payment, replacing Phase 1's manual reconciliation.</t>
+          <t>Combine a drop and a pickup in a single driver trip for efficiency — primarily for Zalora.</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I12" s="25">
         <f>(E12*F12*G12)/H12</f>
         <v/>
       </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>Q4</t>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>TBC</t>
         </is>
       </c>
       <c r="L12" s="19" t="inlineStr">
@@ -4118,83 +3712,10 @@
       </c>
       <c r="O12" s="19" t="inlineStr">
         <is>
-          <t>XD-02 (Phase 1), PG integration</t>
+          <t>Zalora return agreement (Business)</t>
         </is>
       </c>
       <c r="P12" s="19" t="inlineStr">
-        <is>
-          <t>Builds on Phase 1. External payment-gateway dependency plus no PRD yet → confidence low and effort high, so Q4. Sequencing: only start once Phase 1 reconciliation is live and the PG contract/scope is settled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="118" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>XD-09</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Mithril / Driver App</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch &amp; Pick-up (drop + pickup in one trip)</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Combine a drop and a pickup in a single driver trip for efficiency — primarily for Zalora.</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I13" s="22">
-        <f>(E13*F13*G13)/H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>Isumi Karina</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>Zalora return agreement (Business)</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Explicitly deferred in the meeting: not yet a priority because there is no return agreement with Zalora, and no negotiation has started. Blocked on a commercial decision before it can be scoped — Business action needed first, so it can't be scheduled yet.</t>
         </is>

</xml_diff>

<commit_message>
Revise Q3 prioritization from 31 Aug internal meeting + whiteboard (Rev 3)
- Add Short/Medium/Side goal-horizon column across squad tabs (team framing
  from the 31 Aug meeting/whiteboard).
- X-dock: add x-dock-100% umbrella, API integration platform + sandbox,
  Mark-Stock removal / configurable waiting-time-per-stop, outlet-hours master
  data (rider Google Form), inter-hub transit, return dispatch/pickup, and
  timeline media download; expand Retry into Retry + Fail-conditions +
  SLA-defense.
- 4W: add Ops input fields (DN Customer, FO, AGL Route Code); enrich UJP
  (Nexus, spec-control + grounds, master-data research; UJP prioritized over
  P&L).
- Add Tab 7 "Open Questions" capturing unresolved decisions from the 28 & 31
  Aug meetings with owner and what each blocks.
- Refresh Cover legend + September Commitment accordingly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PKPvRHH13fns55VRTHV1kP
</commit_message>
<xml_diff>
--- a/docs/prioritization/q3-2026-prioritization-v1.xlsx
+++ b/docs/prioritization/q3-2026-prioritization-v1.xlsx
@@ -13,6 +13,7 @@
     <sheet name="4. Scheduled Instant — Priority" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. X-dock — Priority" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Push Notif Breakdown" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Open Questions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -591,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -608,7 +609,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Squads: 4W · Scheduled Instant · X-dock   |   PM: Isumi Karina   |   Compiled 31 Aug 2026</t>
+          <t>Squads: 4W · Scheduled Instant · X-dock   |   PM: Isumi Karina   |   Rev 3 · 31 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -620,7 +621,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Consolidate Q3 next-step work across three squads into one prioritized, month-phased backlog. September = the committed slate (P0s + ready quick-wins that unblock live launches: Buku Warung onboarding, 4W rollout, mobile scan-doc). Everything else flows October → Q4. Each squad has its own priority tab, sorted so September items surface first.</t>
+          <t>Consolidate Q3 next-step work across three squads into one prioritized, month-phased backlog. September = the committed slate. Everything else flows October → Q4. Each squad has its own priority tab, sorted so September items surface first. Rev 3 folds in the 31 Aug internal-team meeting + whiteboard.</t>
         </is>
       </c>
     </row>
@@ -632,237 +633,304 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>One priority tab per squad. Reasoning is inline in each tab (the 'Reasoning &amp; sequencing' column) — no separate rationale tab. Driver-App push notifications stay on their own tab (Tab 6). Completed post-release improvements are intentionally excluded — they're already shipped, so they don't need to be carried here.</t>
+          <t>One priority tab per squad. Reasoning is inline (the 'Reasoning &amp; sequencing' column) — no separate rationale tab. Driver-App push notifications stay on Tab 6. Open questions / decisions-needed are on Tab 7. Completed post-release improvements are excluded (already shipped).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Surfaces</t>
+          <t>Goal horizon</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Mithril = internal Ops dashboard · Dash Link = client-facing portal · Driver App = driver mobile app · Back Office / Web = ops tooling · WA = WhatsApp automation · Integration = external client API.</t>
+          <t>Short / Medium / Side — the 31 Aug internal-meeting framing. Short = do now, API + x-dock-100% urgent. Medium = network capability next (transit, return dispatch). Side = opportunistic side-quests (COD, leave-at-outlet, timeline media). Defined by that meeting for X-dock; applied by analogy to 4W / SI.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Priority tiers</t>
+          <t>Surfaces</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>P0 = must-ship this cycle (blocks a live launch / fraud / data-loss) · P1 = high (unblocks scale or removes daily Ops pain) · P2 = important, schedulable · P3 = nice-to-have / deferred.</t>
+          <t>Mithril = internal Ops dashboard · Dash Link = client portal · Driver App = driver mobile app · Back Office / Web = ops tooling · Integration = external client API / sandbox · WA = WhatsApp automation.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Month phasing</t>
+          <t>Priority tiers</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Target month answers 'when does it land'. Sep = committed September slate. Oct / Nov = next in Q3. Q4 = large-scope, blocked-on-business, or exploratory items scoped for later. TBC = awaiting business/leads decision before it can be scheduled.</t>
+          <t>P0 = must-ship this cycle (blocks a live launch / fraud / data-loss) · P1 = high (unblocks scale or removes daily Ops pain) · P2 = important, schedulable · P3 = nice-to-have / deferred.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>RICE scoring</t>
+          <t>Month phasing</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Reach (1-5): trips/users touched per week. Impact (0.5,1,2,3): per-trip severity — data loss/fraud=3; daily Ops friction=2; polish=1; edge=0.5. Confidence (%): certainty the fix delivers the impact (prototype+PRD = higher; no PRD yet = lower). Effort (person-weeks): BE+FE+Mobile combined. Score = (Reach × Impact × Confidence) ÷ Effort. Higher = ship earlier.</t>
+          <t>Sep = committed September slate. Oct / Nov = next in Q3. Q4 = large-scope, blocked-on-business, or exploratory. TBC = awaiting business/leads decision before it can be scheduled.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Readiness</t>
+          <t>RICE scoring</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Signals how fast an item can move. 'Prototype + PRD' = buildable now · 'Prototype only' / 'PRD only' = one artifact missing · 'Draft' = early · 'None — needs PRD/prototype' = requirement gathering first · 'Spike / feasibility' = go/no-go pending. IMPORTANT: every 4W September item still needs PRD + prototype — September for 4W means scope-and-build, so write those PRDs in the first days of the month; the P0s are small (≈1pw each) so this is achievable but not free.</t>
+          <t>Reach (1-5): trips/users touched per week. Impact (0.5,1,2,3): data loss/fraud=3; daily Ops friction=2; polish=1; edge=0.5. Confidence (%): certainty the fix delivers the impact. Effort (person-weeks): BE+FE+Mobile combined. Score = (Reach × Impact × Confidence) ÷ Effort. Higher = ship earlier.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Sort rule</t>
+          <t>Readiness</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Each squad tab is sorted by Target month (Sep → Q4), then Priority (P0 → P3), then Score DESC. So the top of every squad tab is what we're committing to September. Edit RICE inputs and the Score column recalculates; re-sort after edits.</t>
+          <t>'Prototype + PRD' = buildable now · 'Prototype only'/'PRD only' = one artifact missing · 'Draft' = early · 'None — needs PRD/prototype' = requirement gathering first · 'Spike/feasibility' = go/no-go pending. NOTE: every 4W September item still needs PRD + prototype — September for 4W is scope-and-build (write those PRDs in the first days of the month).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Ownership</t>
+          <t>Sort rule</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>PM = Isumi Karina across all items. Engineer ownership is left as 'TBC' — to be assigned. Fill the Engineer column once staffing is confirmed.</t>
+          <t>Each squad tab is sorted by Target month (Sep → Q4), then Priority (P0 → P3), then Score DESC. Edit RICE inputs and the Score column recalculates; re-sort after edits.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Ownership</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>(1) 4W EXIM Post-Release Recap — its RICE next-steps are reused here verbatim with month phasing added. (2) Meeting summary, 28 Aug 2026. (3) Feature &amp; Performance Review — Agustus W2. Where these disagree, the more recent meeting summary wins; open decisions are flagged in each item's reasoning.</t>
+          <t>PM = Isumi Karina across all items. Engineer = 'TBC' (to be assigned; manpower split for short goals is an open item — Tab 7). The 31 Aug meeting named Yogi for R&amp;D / API integration — noted in reasoning, not yet locked in the Engineer column.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>(1) 4W EXIM Post-Release Recap (RICE reused). (2) Meeting summary 28 Aug 2026. (3) Meeting summary 31 Aug 2026 + whiteboard. (4) Feature &amp; Performance Review, Agustus W2. Where they disagree, the more recent meeting wins; open decisions live on Tab 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Rev 3 (31 Aug)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>X-dock: added x-dock-100% umbrella, API integration platform + sandbox, Mark-Stock removal / waiting-time-per-stop, outlet-hours master data, inter-hub transit, return dispatch, timeline media download; expanded Retry into Retry + Fail-conditions + SLA-defense. 4W: added Ops input fields (DN Customer, FO, AGL Route Code); enriched UJP (Nexus / grounds / spec-control, master-data research). Added Tab 7 Open Questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Rev 2 (31 Aug)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Removed as already done: X-dock 'Adjust No. Invoice standardization'; SI 'Phase 2 automated WA confirm loop' and 'Calendar Schedule Metrics'. Removed as cancelled: SI 'NCS API integration'. Merged into one item: SI 'Standardize bulk-upload template' + 'AI CSV header-checker' (two paths to one problem — template committed, AI a feasibility spike). Corrected: all 4W items marked 'needs PRD/prototype' (the recap next-steps are not yet built).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Removed as done: X-dock Adjust No. Invoice; SI Phase 2 WA confirm loop &amp; Calendar metrics. Removed as cancelled: SI NCS API integration. Merged: SI template-standardize + AI header-checker (one item).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Priority swatches</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Must-ship this cycle</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Important, schedulable</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Nice-to-have / deferred</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Month swatches</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Committed September slate</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Next — October</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Later / large-scope / blocked</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Awaiting business decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Goal-horizon swatches</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Do now (31 Aug short goals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Network capability next (medium goals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Opportunistic side-quest</t>
         </is>
       </c>
     </row>
@@ -881,17 +949,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
@@ -904,7 +973,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The committed September slate pulled across all three squads. Full detail &amp; RICE live in each squad tab. PM: Isumi Karina.</t>
+          <t>The committed September slate across all three squads. Full detail &amp; RICE live in each squad tab. PM: Isumi Karina.</t>
         </is>
       </c>
     </row>
@@ -931,26 +1000,31 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Confidence to land Sep</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>Note / dependency</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>X-dock</t>
@@ -958,455 +1032,698 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
+          <t>XD-02</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Retry Shipment + Fail Conditions + SLA defense</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>XD-01, Fail-condition SOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
           <t>XD-01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>X-dock 100% — shipment + route, last-mile, failed conditions</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>In progress — needs PRD</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>XD-07</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>COD Phase 1 — reconciliation</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Prototype + PRD ✓</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>X-dock</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>XD-02</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Retry Shipment</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>XD-03</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>New API integration platform — sandbox, API key, webhook, simulation</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Prototype/simulation exists; timeline revising</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>Sandbox tech spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>XD-06</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Prototype + PRD ✓</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Mobile engineer slot</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>XD-08</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Timeline media download</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD (small)</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Scheduled Instant</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>SI-02</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Pricing per shift</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Prototype + PRD ✓ (pending business)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Business pricing decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Scheduled Instant</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>SI-01</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Exception blast WhatsApp — Noovoleum</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Spike</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>NS-DA-01</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Move completed shipment from Beranda → Riwayat</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>None — needs PRD/prototype</t>
         </is>
       </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H6" s="19" t="inlineStr">
-        <is>
-          <t>Buku Warung onboarding</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>X-dock</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>XD-03</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>NS-MTH-01</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Cancel Shipment (human-error from UJP)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>UJP bridge (import-only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>NS-MTH-02</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Mark as Completed / Mark as Failed (Ops override)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>4W-FLD</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Add Ops input fields: DN Customer, FO, AGL Route Code</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD (small)</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>NS-DL-01</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>EXIM Import/Export tagging (consumer)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Prototype + PRD ✓</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Mobile engineer slot</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Scheduled Instant</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>SI-01</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Exception blast WhatsApp — Noovoleum</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>Spike</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>NS-MTH-03 (Mithril tag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>NS-MTH-03</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>EXIM Import/Export tagging</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="I18" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Scheduled Instant</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>SI-02</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Pricing per shift</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Prototype + PRD ✓ (pending business)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>NS-DA-03</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Push Notifications (full set — see Tab 6)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD (Wave 1)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Business pricing decision</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>NS-DA-01</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Move completed shipment from Beranda → Riwayat</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD/prototype</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>NS-MTH-01</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Cancel Shipment (human-error from UJP)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD/prototype</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>UJP bridge (import-only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>NS-MTH-02</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Mark as Completed / Mark as Failed (Ops override)</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD/prototype</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>NS-DL-01</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>EXIM Import/Export tagging (consumer)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>NS-MTH-03</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>EXIM Import/Export tagging</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD/prototype</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>4W</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>NS-DA-03</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Push Notifications (full set — see Tab 6)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD (Wave 1)</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>NS-MTH-01, NS-MTH-02</t>
         </is>
@@ -1414,8 +1731,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1427,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1441,11 +1758,12 @@
     <col width="7.5" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="58" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="58" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
@@ -1458,7 +1776,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap; Target-month phasing + readiness added. Note: all September items still need PRD/prototype — September is scope-and-build.</t>
+          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap. NEW: Ops input fields (DN Customer, FO, AGL Route Code). All September items still need PRD/prototype — September is scope-and-build.</t>
         </is>
       </c>
     </row>
@@ -1525,31 +1843,37 @@
       </c>
       <c r="L4" s="16" t="inlineStr">
         <is>
+          <t>Goal
+horizon</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="P4" s="16" t="inlineStr">
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>Reasoning &amp; sequencing</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="118" customHeight="1">
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>NS-DA-01</t>
@@ -1596,33 +1920,38 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>None — needs PRD/prototype</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>P0 despite being a 'next-phase' item — it's a live bug surface: drivers can re-fire a completed trip, producing duplicate proof and a confused status timeline. 1pw of Mobile work; makes the interim DA-06 'hide button' hack the real fix. Top RICE score, ships with the September P0 cluster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>P0 despite being a 'next-phase' item — a live bug surface: drivers can re-fire a completed trip, producing duplicate proof and a confused status timeline. 1pw of Mobile work; makes the interim DA-06 'hide button' hack the real fix. Top RICE score, ships with the September P0 cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>NS-MTH-01</t>
@@ -1669,33 +1998,38 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L6" s="19" t="inlineStr">
+      <c r="L6" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>None — needs PRD/prototype</t>
         </is>
       </c>
-      <c r="M6" s="19" t="inlineStr">
+      <c r="N6" s="19" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N6" s="19" t="inlineStr">
+      <c r="O6" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O6" s="19" t="inlineStr">
+      <c r="P6" s="19" t="inlineStr">
         <is>
           <t>UJP bridge (import-only)</t>
         </is>
       </c>
-      <c r="P6" s="19" t="inlineStr">
-        <is>
-          <t>P0 because UJP human-error is a known-recurring issue in feedback. Small state transition + audit reason. Must ship paired with push PN-02 — don't release one without the other or drivers will run cancelled trips.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
+      <c r="Q6" s="19" t="inlineStr">
+        <is>
+          <t>P0 because UJP human-error is a known-recurring issue. Small state transition + audit reason. Must ship paired with push PN-02 — don't release one without the other or drivers will run cancelled trips.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>NS-MTH-02</t>
@@ -1742,51 +2076,56 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>None — needs PRD/prototype</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>P0 because 'driver phone dead' is a real EXIM pattern (long trips, Patimban dead zones). Without it, shipments live IN_DELIVERY forever and billing can't close. Pair with push PN-03.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="118" customHeight="1">
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>NS-DL-01</t>
+          <t>4W-FLD</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Dash Link</t>
+          <t>Mithril / Dash Link / Driver App</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging (consumer)</t>
+          <t>Add Ops input fields: DN Customer, FO, AGL Route Code</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Client-facing filter / column on Dash Link that consumes the Mithril direction tag — no independent work beyond FE render + filter.</t>
+          <t>Capture and display the fields Ops actually needs on 4W shipments — DN Customer, FO, and AGL Route Code — which are missing from the current Create Shipment / workflow forms.</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
@@ -1799,15 +2138,15 @@
         <v>0.85</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I8" s="25">
         <f>(E8*F8*G8)/H8</f>
         <v/>
       </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
@@ -1815,51 +2154,56 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L8" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
+          <t>None — needs PRD (small)</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N8" s="19" t="inlineStr">
+      <c r="O8" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O8" s="19" t="inlineStr">
-        <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
-        </is>
-      </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>TOP quick-win (score 17): 0.5pw because Mithril emits the tag once NS-MTH-03 lands — Dash Link only renders + filters. Client (SwipeRX/AGL Ops) has directly asked to filter by direction. Ship together with, or immediately after, NS-MTH-03 in September.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>Raised by Ops after the internal meeting: the 4W flow lacks the input fields Ops needs to operate and reconcile — DN Customer, FO, and AGL Route Code. Add them to Create Shipment (Mithril), carry through to Shipment details / Dash Link display and the driver flow where relevant, and include them in the print/export templates. Small but blocks clean 4W operations at rollout → September P0. Keys off the AGL Patimban pilot's document/route conventions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>NS-MTH-03</t>
+          <t>NS-DL-01</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Mithril</t>
+          <t>Dash Link</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging</t>
+          <t>EXIM Import/Export tagging (consumer)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Make delivery direction a first-class tag (today it's inferred from stop pattern). Unlocks the Dash Link filter, tracking labels, and Ops reports.</t>
+          <t>Client-facing filter / column on Dash Link that consumes the Mithril direction tag — no independent work beyond FE render + filter.</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
@@ -1869,10 +2213,10 @@
         <v>2</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="22">
         <f>(E9*F9*G9)/H9</f>
@@ -1888,64 +2232,69 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD/prototype</t>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>P1 not P0 — the engine already infers direction, so nothing breaks without it. But it's the unlock for NS-DL-01, NS-DA-02 and future reporting, so schedule it in September right after the P0 cluster to open those quick-wins.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="118" customHeight="1">
+          <t>NS-MTH-03 (Mithril tag)</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>TOP quick-win (score 17): 0.5pw because Mithril emits the tag once NS-MTH-03 lands — Dash Link only renders + filters. Client (SwipeRX/AGL Ops) has directly asked to filter by direction. Ship together with, or immediately after, NS-MTH-03 in September.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>NS-DA-03</t>
+          <t>NS-MTH-03</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Driver App</t>
+          <t>Mithril</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Push Notifications (full set — see Tab 6)</t>
+          <t>EXIM Import/Export tagging</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Zero push today → a driver only learns about a trip by opening the app. Harms on-time gate-in and adds Ops phone-call load. See Tab 6 for the catalogue and per-notif priority.</t>
+          <t>Make delivery direction a first-class tag (today it's inferred from stop pattern). Unlocks the Dash Link filter, tracking labels, and Ops reports.</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="25">
         <f>(E10*F10*G10)/H10</f>
@@ -1961,61 +2310,66 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L10" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD (Wave 1)</t>
+      <c r="L10" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N10" s="19" t="inlineStr">
+      <c r="O10" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O10" s="19" t="inlineStr">
-        <is>
-          <t>NS-MTH-01, NS-MTH-02</t>
-        </is>
-      </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>High reach (every driver, every trip) × high impact (removes Ops WA-broadcast load, cuts late gate-in) × moderate effort (2.5pw). Split into two waves (Tab 6): Wave 1 ships in September with the P0 cluster (PN-02/PN-03 depend on Cancel/Override landing first); Wave 2 follows in October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q10" s="19" t="inlineStr">
+        <is>
+          <t>P1 not P0 — the engine already infers direction, so nothing breaks without it. But it's the unlock for NS-DL-01, NS-DA-02 and future reporting, so schedule it in September right after the P0 cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>4W-NEG</t>
+          <t>NS-DA-03</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Driver App</t>
+          <t>Driver App</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Negative-scenario handling (failure &amp; exception flows)</t>
+          <t>Push Notifications (full set — see Tab 6)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Model the non-happy paths end-to-end: delivery failed, partial delivery, return-to-origin, exception at gate. Today only the happy path is fully handled.</t>
+          <t>Zero push today → a driver only learns about a trip by opening the app. Harms on-time gate-in and adds Ops phone-call load. See Tab 6 for the catalogue and per-notif priority.</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="20" t="n">
         <v>3</v>
       </c>
       <c r="G11" s="21" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H11" s="20" t="n">
         <v>2.5</v>
@@ -2029,56 +2383,61 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD</t>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
+          <t>None — needs PRD (Wave 1)</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>A gap surfaced after the pilot release: the workflow engine handles success cleanly but negative scenarios are ad-hoc. No PRD or prototype yet, so confidence is 0.60 — requirement gathering first, then build. Important for pilot robustness beyond the happy path; targets October so it doesn't compete with the September P0 cluster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="118" customHeight="1">
+          <t>NS-MTH-01, NS-MTH-02</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>High reach × high impact × moderate effort (2.5pw). Split into two waves (Tab 6): Wave 1 ships in September with the P0 cluster (PN-02/PN-03 depend on Cancel/Override landing first); Wave 2 follows in October.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>NS-DA-05</t>
+          <t>4W-NEG</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Driver App</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Local storage + auto-delete (or dedicated logistic app)</t>
+          <t>Negative-scenario handling (failure &amp; exception flows)</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Driver phone dies before evidence syncs → billing evidence lost. Local persistence with server-side reconciliation on reconnect. Alternative under evaluation: a dedicated Dash Logistic app.</t>
+          <t>Model the non-happy paths end-to-end: delivery failed, partial delivery, return-to-origin, exception at gate. Today only the happy path is fully handled.</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
@@ -2088,10 +2447,10 @@
         <v>3</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="I12" s="25">
         <f>(E12*F12*G12)/H12</f>
@@ -2107,36 +2466,41 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L12" s="19" t="inlineStr">
-        <is>
-          <t>Needs arch decision</t>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
+          <t>None — needs PRD</t>
+        </is>
+      </c>
+      <c r="N12" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N12" s="19" t="inlineStr">
+      <c r="O12" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O12" s="19" t="inlineStr">
-        <is>
-          <t>Mobile arch decision (in-app vs new app)</t>
-        </is>
-      </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>P1 but scored below Push: 4pw and it needs an architecture call (enhance the shared app vs. spin a dedicated Dash Logistic app). Do a 1-week spike first, then decide. High impact (prevents evidence loss = prevents billing loss) but confidence is 0.65 until the arch decision is made → October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>A gap surfaced after the pilot release. No PRD or prototype yet (confidence 0.60) — requirement gathering first, then build. Aligns with the X-dock 'failed condition' work (shared fail-reason + evidence patterns). October so it doesn't compete with the September P0 cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>NS-DA-02</t>
+          <t>NS-DA-05</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -2146,33 +2510,33 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging (label on trip card)</t>
+          <t>Local storage + auto-delete (or dedicated logistic app)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>IMPORT / EXPORT badge on Beranda + stepper header — reduces confusion on mixed-lane days.</t>
+          <t>Driver phone dies before evidence syncs → billing evidence lost. Local persistence with server-side reconciliation on reconnect. Alternative: a dedicated Dash Logistic app.</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" s="21" t="n">
-        <v>0.85</v>
+        <v>0.65</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="I13" s="22">
         <f>(E13*F13*G13)/H13</f>
         <v/>
       </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
@@ -2180,36 +2544,41 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
+          <t>Needs arch decision</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
-        </is>
-      </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>0.5pw, purely visual. Impact 1 (not 2): drivers rarely mix directions in one day, so it's a clarity win, not a correctness one. Piggyback on the Mithril tag rollout in October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="118" customHeight="1">
+          <t>Mobile arch decision (in-app vs new app)</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>P1 but scored below Push: 4pw and it needs an architecture call (enhance the shared app vs. spin a dedicated Dash Logistic app). 1-week spike first, then decide. High impact (prevents evidence loss = prevents billing loss) but confidence 0.65 until the arch decision → October.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>NS-DA-04</t>
+          <t>NS-DA-02</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -2219,25 +2588,25 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>Infinix OS: bypass allow-setting workaround</t>
+          <t>EXIM Import/Export tagging (label on trip card)</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Infinix devices block camera/storage permissions by default, preventing Driver App use for a subset of drivers. Vendor-specific fix.</t>
+          <t>IMPORT / EXPORT badge on Beranda + stepper header — reduces confusion on mixed-lane days.</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F14" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="H14" s="23" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="I14" s="25">
         <f>(E14*F14*G14)/H14</f>
@@ -2253,64 +2622,69 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L14" s="19" t="inlineStr">
-        <is>
-          <t>Investigation</t>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
         </is>
       </c>
       <c r="M14" s="19" t="inlineStr">
         <is>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
+        </is>
+      </c>
+      <c r="N14" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N14" s="19" t="inlineStr">
+      <c r="O14" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O14" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>P2 despite high per-user impact — reach is small (only drivers on that OEM). Vendor-specific engineering; ship when an Infinix driver is confirmed in the pilot roster, otherwise defer within October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="118" customHeight="1">
+          <t>NS-MTH-03 (Mithril tag)</t>
+        </is>
+      </c>
+      <c r="Q14" s="19" t="inlineStr">
+        <is>
+          <t>0.5pw, purely visual. Impact 1 (not 2): drivers rarely mix directions in one day, so it's a clarity win. Piggyback on the Mithril tag rollout in October.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>4W-TRK</t>
+          <t>NS-DA-04</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Invoices</t>
+          <t>Driver App</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Tracking invoice 4W</t>
+          <t>Infinix OS: bypass allow-setting workaround</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Import/track 4W invoices by Surat Jalan keyword (4W has no barcode), integrated into the existing Invoices feature.</t>
+          <t>Infinix devices block camera/storage permissions by default, preventing Driver App use for a subset of drivers. Vendor-specific fix.</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G15" s="21" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="I15" s="22">
         <f>(E15*F15*G15)/H15</f>
@@ -2321,69 +2695,74 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="K15" s="14" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>None — post-Sept scope</t>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
-        <is>
-          <t>Invoices feature (existing)</t>
-        </is>
-      </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>Next-phase item from the feature review, scoped after the September rollout so decisions are based on real usage. Connects 4W into the existing Invoices feature; no barcode means it keys off the SJ number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>P2 despite high per-user impact — reach is small (only drivers on that OEM). Ship when an Infinix driver is confirmed in the pilot roster, otherwise defer within October.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>NS-MTH-04</t>
+          <t>4W-TRK</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Mithril</t>
+          <t>Mithril / Invoices</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Full sistem UJP — migrate UJP → Mithril (native module)</t>
+          <t>Tracking invoice 4W</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Bring UJP native into Mithril (today it's a separate system with an import-only bridge). Removes double-entry, closes the fraud loop, connects to Basecamp API for finance uang-jalan approval, and enables end-to-end reporting.</t>
+          <t>Import/track 4W invoices by Surat Jalan keyword (4W has no barcode), integrated into the existing Invoices feature.</t>
         </is>
       </c>
       <c r="E16" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" s="24" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I16" s="25">
         <f>(E16*F16*G16)/H16</f>
@@ -2399,64 +2778,69 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="L16" s="19" t="inlineStr">
-        <is>
-          <t>None — needs PRD</t>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
         </is>
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
+          <t>None — post-Sept scope</t>
+        </is>
+      </c>
+      <c r="N16" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N16" s="19" t="inlineStr">
+      <c r="O16" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O16" s="19" t="inlineStr">
-        <is>
-          <t>Mithril auth + role model, Basecamp API</t>
-        </is>
-      </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Largest scope item (6pw) and the user-flagged 'sistem UJP' — no PRD or prototype yet. P2 not P1 because the import-only bridge already handles the fraud gate for Phase 0. Real value is Ops efficiency + closing double-entry + native finance approval; schedule after the pilot is stable and Phase 0 EXIM is proven.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="118" customHeight="1">
+          <t>Invoices feature (existing)</t>
+        </is>
+      </c>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>Next-phase item from the feature review, scoped after the September rollout so decisions are based on real usage. Connects 4W into the existing Invoices feature; no barcode means it keys off the SJ number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>4W-FLT</t>
+          <t>NS-MTH-04</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Driver App / Fleet</t>
+          <t>Mithril / Nexus</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Integrasi Fleet — pre-trip QR scan</t>
+          <t>Full sistem UJP — migrate UJP → Mithril (native module)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Driver scans a vehicle QR at pre-trip so they take the assigned vehicle; the scan result syncs to the Fleet system.</t>
+          <t>Bring UJP native into Mithril (today it's a separate system in Nexus with an import-only bridge). Removes double-entry, closes the fraud loop, and enables end-to-end finance reporting.</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" s="21" t="n">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="I17" s="22">
         <f>(E17*F17*G17)/H17</f>
@@ -2472,27 +2856,110 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD + master-data research</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>spec control + 'grounds', Basecamp API</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>Largest scope item (6pw) and the user-flagged 'sistem UJP'. 31 Aug confirmed UJP as the CORE for 4-wheels and prioritized it over P&amp;L (P&amp;L can stay in the existing system for now). UJP lives in Nexus and must integrate with spec control and 'grounds' (which own auto-P&amp;L + control); upload needs master data from several sources → research first. P&amp;L / gross-margin / payroll / 'kois' automation is a later side-quest once all clients use full shipment. Schedule after the pilot is stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>4W-FLT</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Driver App / Fleet</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Integrasi Fleet — pre-trip QR scan</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Driver scans a vehicle QR at pre-trip so they take the assigned vehicle; the scan result syncs to the Fleet system.</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H18" s="23" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I18" s="25">
+        <f>(E18*F18*G18)/H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
         <is>
           <t>None — post-Sept scope</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="N18" s="19" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="O18" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr">
+      <c r="P18" s="19" t="inlineStr">
         <is>
           <t>Fleet system</t>
         </is>
       </c>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="Q18" s="19" t="inlineStr">
         <is>
           <t>Cross-system dependency on Fleet. Next-phase, scoped after the September rollout review. Ensures driver-vehicle assignment integrity; lower confidence until the Fleet-side contract is confirmed.</t>
         </is>
@@ -2500,8 +2967,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2513,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2527,11 +2994,12 @@
     <col width="7.5" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="58" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="58" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
@@ -2544,7 +3012,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scheduled Instant — rider scheduling &amp; shipment intake. September = Noovoleum WA exception + pricing per shift. Removed: NCS API integration (cancelled), Phase 2 WA confirm loop &amp; Calendar metrics (already done).</t>
+          <t>Scheduled Instant — rider scheduling &amp; shipment intake. September = Noovoleum WA exception + pricing per shift.</t>
         </is>
       </c>
     </row>
@@ -2611,31 +3079,37 @@
       </c>
       <c r="L4" s="16" t="inlineStr">
         <is>
+          <t>Goal
+horizon</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="P4" s="16" t="inlineStr">
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>Reasoning &amp; sequencing</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="118" customHeight="1">
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>SI-02</t>
@@ -2682,33 +3156,38 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Prototype + PRD ✓ (pending business)</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Business pricing decision</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>Prototype + PRD are ready; the only blocker is the commercial pricing decision. Raise it in the Mon 1 Sept priority meeting with Pak Harina; once decided it lands in September. Unlocks correct billing for dedicated-manpower clients.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>Prototype + PRD ready; the only blocker is the commercial pricing decision. Raise it in the Mon 1 Sept priority meeting with Pak Harina; once decided it lands in September. Unlocks correct billing for dedicated-manpower clients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>SI-01</t>
@@ -2755,33 +3234,38 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L6" s="19" t="inlineStr">
+      <c r="L6" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>Spike</t>
         </is>
       </c>
-      <c r="M6" s="19" t="inlineStr">
+      <c r="N6" s="19" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N6" s="19" t="inlineStr">
+      <c r="O6" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O6" s="19" t="inlineStr">
+      <c r="P6" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="19" t="inlineStr">
+      <c r="Q6" s="19" t="inlineStr">
         <is>
           <t>Client commitment, currently being spiked by engineering. Small in scope but client-blocking, so it rides with the September P0 slate.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="118" customHeight="1">
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>SI-03</t>
@@ -2828,33 +3312,38 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>PRD only</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>Replaces a manual Ops workaround with a native view. Useful but not launch-blocking → October.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="118" customHeight="1">
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>SI-04</t>
@@ -2872,7 +3361,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>One initiative, two paths to the same goal — let clients self-upload orders without the Ops team, cutting human error. Path A (committed): standardize the bulk-upload template header so uploads are consistent across clients. Path B (spike): an AI that auto-validates arbitrary/dynamic client CSV headers.</t>
+          <t>One initiative, two paths to the same goal — let clients self-upload orders without the Ops team, cutting human error. Path A (committed): standardize the bulk-upload template header. Path B (spike): an AI that auto-validates arbitrary/dynamic client CSV headers.</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
@@ -2901,33 +3390,38 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L8" s="19" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M8" s="19" t="inlineStr">
         <is>
           <t>Draft template (AI = feasibility spike)</t>
         </is>
       </c>
-      <c r="M8" s="19" t="inlineStr">
+      <c r="N8" s="19" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N8" s="19" t="inlineStr">
+      <c r="O8" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O8" s="19" t="inlineStr">
+      <c r="P8" s="19" t="inlineStr">
         <is>
           <t>Speaker 1 CSV analysis</t>
         </is>
       </c>
-      <c r="P8" s="19" t="inlineStr">
-        <is>
-          <t>These are two solutions to one problem, so they're tracked as one item. A draft template already exists (Path A). The meeting explored the AI header-checker (Path B) but engineering judged the effort very large — client templates are highly dynamic, manual validation is still needed up front, and pulling supporting data (e.g. customer records) is hard. Decision: commit to standardizing the template first; run the AI checker only as a time-boxed feasibility spike whose go/no-go rests on Speaker 1's analysis of NCS's sample CSV. If the AI path isn't feasible, we keep the standardized template and drop the AI work. Confidence held at 0.55 because the committed scope (template) is clear but the AI upside is unproven.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="118" customHeight="1">
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>Two solutions to one problem, tracked as one item; appears on the 31 Aug board as side-quest 'shipment AI upload?'. A draft template exists (Path A). The 28 Aug meeting judged the AI checker (Path B) very high-effort — client templates are dynamic, manual validation is still needed up front, supporting data is hard to pull. Decision: commit to the template first; run the AI checker only as a time-boxed spike whose go/no-go rests on Speaker 1's analysis of NCS's sample CSV (Tab 7). Confidence 0.55: committed scope clear, AI upside unproven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>SI-05</t>
@@ -2974,27 +3468,32 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>TBC — business / leads</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Business &amp; Leads scope</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>Detail and context are incomplete — still TBC with Business &amp; Leads. Cannot be scoped or scheduled until they define the requirement, so it sits outside the month plan for now.</t>
         </is>
@@ -3002,8 +3501,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3015,7 +3514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3029,11 +3528,12 @@
     <col width="7.5" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="58" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="58" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
@@ -3046,7 +3546,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cross-docking — goal: move all cross-dock clients to the new app. September = COD Phase 1, retry shipment, scan-doc/leave-at-outlet. Removed: Adjust No. Invoice standardization (already done).</t>
+          <t>Cross-docking — 31 Aug internal meeting: Short goals (x-dock 100%, retry+fail-conditions, API platform), Medium goals (transit, return dispatch), Side quests (COD, leave-at-outlet, timeline media).</t>
         </is>
       </c>
     </row>
@@ -3113,31 +3613,37 @@
       </c>
       <c r="L4" s="16" t="inlineStr">
         <is>
+          <t>Goal
+horizon</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="P4" s="16" t="inlineStr">
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>Reasoning &amp; sequencing</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="118" customHeight="1">
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>XD-02</t>
@@ -3150,12 +3656,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Retry Shipment</t>
+          <t>Retry Shipment + Fail Conditions + SLA defense</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Auto-retry failed deliveries (e.g. pharmacy closed) with a structured re-attempt instead of manual re-create. Needed across many clients — Buku Warung and SwipeRX called out.</t>
+          <t>When a delivery can't complete (outlet/pharmacy closed, no time left), the driver logs a recorded fail reason with field evidence instead of a new shipment being created blindly. Fail conditions + evidence let Dash defend its SLA against unfair client penalties.</t>
         </is>
       </c>
       <c r="E5" s="20" t="n">
@@ -3184,33 +3690,38 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>None — needs PRD/prototype</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>Buku Warung onboarding</t>
-        </is>
-      </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Top of the meeting's priority list and highest reach (multi-client). But no PRD or prototype yet, so confidence is held at 0.70: run requirement gathering in the first week of September, then build. Buku Warung targets go-live W2–W3 September with API integration accepted as not-ready-at-launch (~1 month grace) — retry is what keeps that onboarding reliable, so it stays a September P0 even though the build may finish end-of-month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+          <t>XD-01, Fail-condition SOP</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>The 31 Aug meeting sharpened this into three linked parts: (a) Retry instead of blind re-create; (b) Fail Conditions (time not possible, outlet closed, …) each needing field evidence, e.g. a photo of the closed outlet; (c) SLA rebuttal — a valid fail (outlet closed) must not count against Dash's SLA with the client. Short goal 1.1, 'segera setelah item sebelumnya'. Highest reach (Buku Warung, SwipeRX). Still needs a PRD and a fail-condition SOP (Tab 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>XD-01</t>
@@ -3218,30 +3729,30 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Back Office</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>COD Phase 1 — reconciliation</t>
+          <t>X-dock 100% — shipment + route, last-mile, failed conditions</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Record and reconcile Cash-on-Delivery collected per shipment (Zalora). Scope is reconciliation only — no payment-gateway link yet.</t>
+          <t>Get every cross-docking client fully onto the new app end-to-end: shipment + route assignment, last-mile coverage, and failed-condition handling. The umbrella short goal.</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="23" t="n">
-        <v>2</v>
-      </c>
       <c r="G6" s="24" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I6" s="25">
         <f>(E6*F6*G6)/H6</f>
@@ -3257,61 +3768,66 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L6" s="19" t="inlineStr">
-        <is>
-          <t>Prototype + PRD ✓</t>
+      <c r="L6" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M6" s="19" t="inlineStr">
         <is>
+          <t>In progress — needs PRD</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N6" s="19" t="inlineStr">
+      <c r="O6" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O6" s="19" t="inlineStr">
+      <c r="P6" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="19" t="inlineStr">
-        <is>
-          <t>Active focus per the meeting: one engineer paused 'upload performance' to concentrate on COD, working to Albert's PRD. Prototype + PRD are ready and scope is deliberately narrow (reconciliation), so it fits September. Phase 2 (payment-gateway QRIS auto-check) is split out as XD-07.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
+      <c r="Q6" s="19" t="inlineStr">
+        <is>
+          <t>Short goal #1 from the 31 Aug internal meeting ('x-dock 100%'). This is the parent effort: shipment + route works for every client, last-mile is covered, and failed conditions are captured (not silently re-created). Retry Shipment (XD-02) is its immediate follow-on (meeting item 1.1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>XD-03</t>
+          <t>XD-07</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Driver App (Mobile)</t>
+          <t>Mithril / Back Office</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
+          <t>COD Phase 1 — reconciliation</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Driver handles multiple invoices in one outlet visit, plus a 'leave at outlet' option with a scanned blank-document (BAST) as proof.</t>
+          <t>Record and reconcile Cash-on-Delivery collected per shipment (Zalora). Reconciliation only — no payment-gateway link yet.</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="H7" s="20" t="n">
         <v>1.5</v>
@@ -3320,9 +3836,9 @@
         <f>(E7*F7*G7)/H7</f>
         <v/>
       </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
@@ -3330,137 +3846,147 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Prototype + PRD ✓</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>Mobile engineer slot</t>
-        </is>
-      </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>Prototype + PRD ready and a mobile engineer is confirmed to pick it up Thursday 3 September — a clean September win. Cuts failed-visit re-dispatch and matches how drivers actually work outlets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Whiteboard side quest #1. Active focus per the 28 Aug meeting: one engineer paused 'upload performance' to concentrate on COD, working to Albert's PRD. Prototype + PRD ready and scope is narrow, so it fits September. Phase 2 (payment-gateway QRIS auto-check) is XD-14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>XD-04</t>
+          <t>XD-03</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Driver App</t>
+          <t>Integration / Dash Link</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Shipment Bypass Hub — SwipeRX</t>
+          <t>New API integration platform — sandbox, API key, webhook, simulation</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Rider rides the van from the Tempe warehouse straight to the pharmacy, bypassing the Dash hub. Uses Create Shipment with origin = client hub.</t>
+          <t>A reusable API integration capability so clients can integrate order intake — sandbox (auto-single-run), API keys, webhooks, developer mode — instead of one-off manual integrations.</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="23" t="n">
-        <v>2</v>
-      </c>
       <c r="G8" s="24" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="I8" s="25">
         <f>(E8*F8*G8)/H8</f>
         <v/>
       </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L8" s="19" t="inlineStr">
-        <is>
-          <t>Prototype ready</t>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
+          <t>Prototype/simulation exists; timeline revising</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N8" s="19" t="inlineStr">
+      <c r="O8" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Prototype is ready, status pending. SwipeRX-specific and not blocking any September launch, so schedule right after the P0 cluster in October.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="118" customHeight="1">
+          <t>Sandbox tech spec</t>
+        </is>
+      </c>
+      <c r="Q8" s="19" t="inlineStr">
+        <is>
+          <t>Short goal #2 ('new api integration'), prioritized because API demand is urgent (31 Aug). Distinct from the cancelled NCS-specific integration — this is the general platform: sandbox focused on Dash Link, developer mode, GitHub repo, auto-run so API + UI run automatically. Prototype/simulation already exists; timeline being revised. Yogi = R&amp;D / integration lead per the meeting (Engineer still TBC in the column). Spans Sep→Oct; sandbox spec is an open item (Tab 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>XD-05</t>
+          <t>XD-06</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Mithril</t>
+          <t>Driver App (Mobile)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Filter client X-dock in Schedule menu</t>
+          <t>Multi-invoice per visit + scan blank document / leave at outlet</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>X-dock shares the Schedule calendar (default filter is currently Scheduled Instant); it needs a per-squad filter. The X-dock calendar stays empty until requirement gathering fills it.</t>
+          <t>Driver handles multiple invoices in one outlet visit, plus a 'leave at outlet' option with a scanned blank-document (BAST) as proof.</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="21" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I9" s="22">
         <f>(E9*F9*G9)/H9</f>
@@ -3471,56 +3997,61 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>PRD partial — needs detail</t>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
+          <t>Prototype + PRD ✓</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Detail depends on requirement gathering that hasn't happened; low urgency next to the P0 cluster, so October. The filter itself is small — the calendar content behind it is the real open question.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="118" customHeight="1">
+          <t>Mobile engineer slot</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Prototype + PRD ready and a mobile engineer picks it up Thursday 3 September — a clean September win. Whiteboard side quest #3 ('tinggal SJ'). Cuts failed-visit re-dispatch and matches how drivers work outlets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>XD-06</t>
+          <t>XD-08</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Dash Link</t>
+          <t>Mithril</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Performance invoice — POV outlet</t>
+          <t>Timeline media download</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Invoice performance from the outlet's point of view (Logistic Mithril &amp; Dash Link). Primarily a client request.</t>
+          <t>Download media (proof photos) from the shipment timeline in Mithril, for client evidence sharing.</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
@@ -3530,10 +4061,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>0.85</v>
+        <v>0.7</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="25">
         <f>(E10*F10*G10)/H10</f>
@@ -3544,56 +4075,61 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="L10" s="19" t="inlineStr">
-        <is>
-          <t>Prototype + PRD ✓ (paused)</t>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
         </is>
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
+          <t>None — needs PRD (small)</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N10" s="19" t="inlineStr">
+      <c r="O10" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O10" s="19" t="inlineStr">
+      <c r="P10" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P10" s="19" t="inlineStr">
-        <is>
-          <t>Ready but deliberately paused: per the meeting, the engineer moved off 'upload performance' onto COD. Resume in October once COD Phase 1 is stable. Low reach (reporting view), so P2 despite being buildable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="118" customHeight="1">
+      <c r="Q10" s="19" t="inlineStr">
+        <is>
+          <t>Whiteboard side quest #4 ('timeline media download → Mithril'), target ~9 September. Small; download proof media from the timeline. Schedule opportunistically inside September; low effort so it doesn't threaten the short-goal spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>XD-07</t>
+          <t>XD-05</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Back Office + PG</t>
+          <t>Back Office / Data</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>COD Phase 2 — Payment Gateway QRIS auto-check</t>
+          <t>Master data — outlet goods-receiving hours (rider Google Form)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Connect COD to the Payment Gateway to auto-verify QRIS payment, replacing Phase 1's manual reconciliation.</t>
+          <t>Reliable master data of each outlet's goods-receiving hours, to drive waiting-time and prioritization.</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
@@ -3603,55 +4139,60 @@
         <v>2</v>
       </c>
       <c r="G11" s="21" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I11" s="22">
         <f>(E11*F11*G11)/H11</f>
         <v/>
       </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K11" s="14" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>None — needs PRD</t>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
+          <t>None — needs process</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>XD-01 (Phase 1), PG integration</t>
-        </is>
-      </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Builds on Phase 1. External payment-gateway dependency plus no PRD yet → confidence low and effort high, so Q4. Sequencing: only start once Phase 1 reconciliation is live and the PG contract/scope is settled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="118" customHeight="1">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>31 Aug: Google Maps scraping is inaccurate for receiving hours. Instead collect via a rider Google Form → spreadsheet → master data, focused on client outlets first. Low-effort and it unblocks XD-04, so high score. Mostly an Ops data-collection process + a small import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>XD-08</t>
+          <t>XD-09</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
@@ -3661,70 +4202,543 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Dispatch &amp; Pick-up (drop + pickup in one trip)</t>
+          <t>Shipment Bypass Hub — SwipeRX</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Combine a drop and a pickup in a single driver trip for efficiency — primarily for Zalora.</t>
+          <t>Rider rides the van from the Tempe warehouse straight to the pharmacy, bypassing the Dash hub. Uses Create Shipment with origin = client hub.</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I12" s="25">
         <f>(E12*F12*G12)/H12</f>
         <v/>
       </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="K12" s="15" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M12" s="19" t="inlineStr">
+        <is>
+          <t>Prototype ready</t>
+        </is>
+      </c>
+      <c r="N12" s="19" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O12" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="L12" s="19" t="inlineStr">
+      <c r="P12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>Prototype ready, status pending. SwipeRX-specific and not blocking any September launch, so October after the short-goal cluster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>XD-04</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Mithril / Dispatch</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Remove 'Mark Stock' → configurable waiting-time-per-stop + outlet-hour prioritization</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Ops shouldn't manage stock via 'Mark Stock'. Replace it with a per-client configurable waiting-time-per-stop and order prioritization driven by outlet operational hours.</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="22">
+        <f>(E13*F13*G13)/H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>None — needs PRD</t>
         </is>
       </c>
-      <c r="M12" s="19" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="N12" s="19" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="O12" s="19" t="inlineStr">
-        <is>
-          <t>Zalora return agreement (Business)</t>
-        </is>
-      </c>
-      <c r="P12" s="19" t="inlineStr">
-        <is>
-          <t>Explicitly deferred in the meeting: not yet a priority because there is no return agreement with Zalora, and no negotiation has started. Blocked on a commercial decision before it can be scoped — Business action needed first, so it can't be scheduled yet.</t>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>XD-05 (outlet-hours master data)</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>31 Aug: 'Mark Stock' exists only because capacity is inaccurate, time is tight, and waiting-time-per-stop isn't modeled. Fix the root cause — configurable waiting time per stop (per client) + prioritize orders by outlet operational hours (whiteboard: outlet operational hour → waiting time per stop → clients). Removes a recurring Ops chore; depends on the outlet-hours master data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>XD-10</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Mithril</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Filter client X-dock in Schedule menu</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>X-dock shares the Schedule calendar (default filter is Scheduled Instant); it needs a per-squad filter. The X-dock calendar stays empty until requirement gathering fills it.</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="25">
+        <f>(E14*F14*G14)/H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L14" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M14" s="19" t="inlineStr">
+        <is>
+          <t>PRD partial — needs detail</t>
+        </is>
+      </c>
+      <c r="N14" s="19" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O14" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q14" s="19" t="inlineStr">
+        <is>
+          <t>Detail depends on requirement gathering that hasn't happened; low urgency next to the short-goal cluster, so October. The filter is small — the calendar content behind it is the real open question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>XD-11</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Mithril / Dash Link</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Performance invoice — POV outlet</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Invoice performance from the outlet's point of view (Logistic Mithril &amp; Dash Link). Primarily a client request.</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="22">
+        <f>(E15*F15*G15)/H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Prototype + PRD ✓ (paused)</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Ready but deliberately paused: per the meeting the engineer moved off 'upload performance' onto COD. Resume in October once COD Phase 1 is stable. Low reach (reporting view), so P2 despite being buildable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>XD-12</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Mithril / Ops</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Transit antar-hub (inter-hub transit)</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Route long-distance orders between hubs via scheduled transit: pickup region → back to hub → transit → deliver to destination. Run manually first.</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H16" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="25">
+        <f>(E16*F16*G16)/H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="M16" s="19" t="inlineStr">
+        <is>
+          <t>Manual first — needs PRD</t>
+        </is>
+      </c>
+      <c r="N16" s="19" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O16" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P16" s="19" t="inlineStr">
+        <is>
+          <t>Dispatch schedule per hub</t>
+        </is>
+      </c>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>31 Aug medium goal #1. Transit times morning/noon/night (morning &amp; noon most important); tightly coupled to the dispatch schedule (e.g. dispatch 9am → transit must leave by 7am). Large coverage and scheduling-sensitive, so start manual and systematize later. Open risk: partners without an app keep transit manual — a mitra queueing tool is an open question (Tab 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>XD-13</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Mithril / Driver App</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Return dispatch / pickup (hub-to-hub) → feeds transit</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Let a hub receive a shipment from a desk to another hub, and combine a drop + pickup in one driver trip. Feeds the inter-hub transit flow.</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I17" s="22">
+        <f>(E17*F17*G17)/H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>XD-12 (transit), Zalora return agreement (Business)</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>31 Aug medium goal #2. Broader than the earlier Zalora dispatch+pickup: return dispatch/pickup lets a hub receive shipment from desk → another hub, which must align with the transit flow. The pickup-combine part still needs the Zalora return agreement (no negotiation started). Medium goal → Q4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>XD-14</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Mithril / Back Office + PG</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>COD Phase 2 — Payment Gateway QRIS auto-check</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Connect COD to the Payment Gateway to auto-verify QRIS payment, replacing Phase 1's manual reconciliation.</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H18" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="25">
+        <f>(E18*F18*G18)/H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD</t>
+        </is>
+      </c>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O18" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P18" s="19" t="inlineStr">
+        <is>
+          <t>XD-07 (Phase 1), PG integration</t>
+        </is>
+      </c>
+      <c r="Q18" s="19" t="inlineStr">
+        <is>
+          <t>Builds on Phase 1. External payment-gateway dependency plus no PRD yet → confidence low and effort high, so Q4. Start only once Phase 1 reconciliation is live and the PG contract/scope is settled.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3759,7 +4773,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kept on its own tab (per structure). Batched in 2 waves. Wave 1 = trip-critical (blocks driver from acting) — ships Sep with 4W P0 cluster. Wave 2 = supportive — Oct.</t>
+          <t>Kept on its own tab. 2 waves. Wave 1 = trip-critical (blocks driver from acting) — ships Sep with the 4W P0 cluster. Wave 2 = supportive — Oct.</t>
         </is>
       </c>
     </row>
@@ -4106,4 +5120,396 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="31.5" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Open Questions &amp; Decisions Needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="21.75" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Unresolved items from the 28 &amp; 31 Aug meetings that block or shape prioritized work. Resolve to unlock the linked items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Question / decision</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Blocks</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Needed by</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>OQ-01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Fail-condition SOP + evidence format for Retry Shipment — full list of fail reasons and what proof each needs (e.g. photo of closed outlet).</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Product + Ops</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>XD-02 (Retry + SLA defense)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Early Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>OQ-02</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Manpower split for short goals — who owns x-dock 100%, Retry, and the API platform; individual assignments.</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>All / X-dock</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Leads (next meeting)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>XD-01, XD-02, XD-03 land dates</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Early Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>OQ-03</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Sandbox technical spec + revised API timeline — scope, environment, auto-run pipeline; GitHub repo.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>X-dock / Eng</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Eng (Yogi, R&amp;D)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>XD-03 (API platform)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>OQ-04</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Pricing per shift — commercial decision (dedicated manpower / daily-flat rates).</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Scheduled Instant</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Business (Pak Harina, Mon 1 Sep)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>SI-02 (Pricing per shift)</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>1 Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>OQ-05</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Transit scheduling detail — exact transit times &amp; frequency per hub; dispatch schedule alignment (e.g. dispatch 9am → transit by 7am).</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>XD-12 (inter-hub transit)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Q4 scoping</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>OQ-06</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Mitra queueing tool — partners without an app; does Faktual Capital / HAPI / LASMAN replace the IT-Mitra role, or does transit stay manual?</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Business / IT</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>XD-12 (transit rollout)</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Q4 scoping</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>OQ-07</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Zalora return agreement — commercial agreement for return dispatch/pickup (no negotiation started yet).</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>X-dock</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>XD-13 (return dispatch/pickup)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Before Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>OQ-08</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>AI CSV upload feasibility — Speaker 1 to analyze NCS sample CSV template &amp; logic; go/no-go on the AI header-checker.</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Scheduled Instant</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Product + Eng (Speaker 1)</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>SI-04 (AI spike path)</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>OQ-09</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>UJP upload master-data sources — identify every source needed to upload UJP; integration with spec control &amp; 'grounds'.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Eng + Ops</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>NS-MTH-04 (UJP native)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Q4 scoping</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>OQ-10</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>4W Ops input fields — confirm exact definition &amp; source of DN Customer, FO, and AGL Route Code (validation rules, where they display).</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Ops + Product</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>4W-FLD (Ops input fields)</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Early Sep</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4W EXIM tagging selector at Create Shipment (per-client default workflow)
New 4W item 4W-TAG: an Export/Import/None tag selector at Create Shipment that
drives a different default workflow per client (None = general default),
extending the first-class EXIM tag (NS-MTH-03) into an Ops-facing selector and
building on the shipped "one client -> multiple pickup workflows" improvement.
P0/September. Add matching open question OQ-11 (confirm the default workflow
mapped to each tag per client).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PKPvRHH13fns55VRTHV1kP
</commit_message>
<xml_diff>
--- a/docs/prioritization/q3-2026-prioritization-v1.xlsx
+++ b/docs/prioritization/q3-2026-prioritization-v1.xlsx
@@ -949,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1596,17 +1596,17 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>NS-DL-01</t>
+          <t>4W-TAG</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging (consumer)</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>EXIM tagging selector (Export / Import / None) → per-client default workflow</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
+          <t>None — needs PRD (small)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
+          <t>NS-MTH-03 (first-class EXIM tag), 4W-FLD</t>
         </is>
       </c>
     </row>
@@ -1643,12 +1643,12 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>NS-MTH-03</t>
+          <t>NS-DL-01</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging</t>
+          <t>EXIM Import/Export tagging (consumer)</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>None — needs PRD/prototype</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="I18" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NS-MTH-03 (Mithril tag)</t>
         </is>
       </c>
     </row>
@@ -1690,40 +1690,87 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
+          <t>NS-MTH-03</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>EXIM Import/Export tagging</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>None — needs PRD/prototype</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
           <t>NS-DA-03</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>Push Notifications (full set — see Tab 6)</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>Short</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>None — needs PRD (Wave 1)</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I20" s="19" t="inlineStr">
         <is>
           <t>NS-MTH-01, NS-MTH-02</t>
         </is>
@@ -1744,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1776,7 +1823,7 @@
     <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap. NEW: Ops input fields (DN Customer, FO, AGL Route Code). All September items still need PRD/prototype — September is scope-and-build.</t>
+          <t>4W (roda-4) — pilot AGL Patimban. RICE reused from the Post-Release Recap. NEW at Create Shipment: Ops input fields (DN Customer, FO, AGL Route Code) + EXIM tagging selector (Export/Import/None) → per-client default workflow. All September items still need PRD/prototype — September is scope-and-build.</t>
         </is>
       </c>
     </row>
@@ -2188,22 +2235,22 @@
     <row r="9" ht="120" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>NS-DL-01</t>
+          <t>4W-TAG</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Dash Link</t>
+          <t>Mithril / Create Shipment</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging (consumer)</t>
+          <t>EXIM tagging selector (Export / Import / None) → per-client default workflow</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Client-facing filter / column on Dash Link that consumes the Mithril direction tag — no independent work beyond FE render + filter.</t>
+          <t>At Create Shipment, Ops picks a tag — Export / Import / None (None = general clients) — and the system loads a different default workflow per client per tag, instead of Ops re-picking the flow every time.</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
@@ -2216,15 +2263,15 @@
         <v>0.85</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="I9" s="22">
         <f>(E9*F9*G9)/H9</f>
         <v/>
       </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr">
@@ -2239,7 +2286,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
+          <t>None — needs PRD (small)</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -2254,34 +2301,34 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
+          <t>NS-MTH-03 (first-class EXIM tag), 4W-FLD</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>TOP quick-win (score 17): 0.5pw because Mithril emits the tag once NS-MTH-03 lands — Dash Link only renders + filters. Client (SwipeRX/AGL Ops) has directly asked to filter by direction. Ship together with, or immediately after, NS-MTH-03 in September.</t>
+          <t>Raised by Ops alongside the input fields. Extends NS-MTH-03: that item makes direction a first-class tag (today it's inferred from stop pattern); this exposes the tag as a manual selector at Create Shipment (Export / Import / None) and wires each value to a client's default workflow — so an Export order for a client auto-loads its Export flow, Import its Import flow, and None a general default. Builds on the already-shipped 'one client → multiple pickup workflows' improvement (MTH-01). Small but it's what makes per-client, per-direction workflows usable by Ops at intake → September P0. Pair with 4W-FLD (both are Create Shipment additions).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>NS-MTH-03</t>
+          <t>NS-DL-01</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Mithril</t>
+          <t>Dash Link</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging</t>
+          <t>EXIM Import/Export tagging (consumer)</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Make delivery direction a first-class tag (today it's inferred from stop pattern). Unlocks the Dash Link filter, tracking labels, and Ops reports.</t>
+          <t>Client-facing filter / column on Dash Link that consumes the Mithril direction tag — no independent work beyond FE render + filter.</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
@@ -2291,10 +2338,10 @@
         <v>2</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="25">
         <f>(E10*F10*G10)/H10</f>
@@ -2317,7 +2364,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>None — needs PRD/prototype</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="N10" s="19" t="inlineStr">
@@ -2332,47 +2379,47 @@
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NS-MTH-03 (Mithril tag)</t>
         </is>
       </c>
       <c r="Q10" s="19" t="inlineStr">
         <is>
-          <t>P1 not P0 — the engine already infers direction, so nothing breaks without it. But it's the unlock for NS-DL-01, NS-DA-02 and future reporting, so schedule it in September right after the P0 cluster.</t>
+          <t>TOP quick-win (score 17): 0.5pw because Mithril emits the tag once NS-MTH-03 lands — Dash Link only renders + filters. Client (SwipeRX/AGL Ops) has directly asked to filter by direction. Ship together with, or immediately after, NS-MTH-03 in September.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>NS-DA-03</t>
+          <t>NS-MTH-03</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Driver App</t>
+          <t>Mithril</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Push Notifications (full set — see Tab 6)</t>
+          <t>EXIM Import/Export tagging</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Zero push today → a driver only learns about a trip by opening the app. Harms on-time gate-in and adds Ops phone-call load. See Tab 6 for the catalogue and per-notif priority.</t>
+          <t>Make delivery direction a first-class tag (today it's inferred from stop pattern). Unlocks the Dash Link filter, tracking labels, and Ops reports.</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
         <v>5</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" s="21" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I11" s="22">
         <f>(E11*F11*G11)/H11</f>
@@ -2395,7 +2442,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>None — needs PRD (Wave 1)</t>
+          <t>None — needs PRD/prototype</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -2410,44 +2457,44 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>NS-MTH-01, NS-MTH-02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>High reach × high impact × moderate effort (2.5pw). Split into two waves (Tab 6): Wave 1 ships in September with the P0 cluster (PN-02/PN-03 depend on Cancel/Override landing first); Wave 2 follows in October.</t>
+          <t>P1 not P0 — the engine already infers direction, so nothing breaks without it. But it's the unlock for NS-DL-01, NS-DA-02 and future reporting, so schedule it in September right after the P0 cluster.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>4W-NEG</t>
+          <t>NS-DA-03</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Driver App</t>
+          <t>Driver App</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Negative-scenario handling (failure &amp; exception flows)</t>
+          <t>Push Notifications (full set — see Tab 6)</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Model the non-happy paths end-to-end: delivery failed, partial delivery, return-to-origin, exception at gate. Today only the happy path is fully handled.</t>
+          <t>Zero push today → a driver only learns about a trip by opening the app. Harms on-time gate-in and adds Ops phone-call load. See Tab 6 for the catalogue and per-notif priority.</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>3</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H12" s="23" t="n">
         <v>2.5</v>
@@ -2461,9 +2508,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K12" s="12" t="inlineStr">
-        <is>
-          <t>Oct</t>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>Sep</t>
         </is>
       </c>
       <c r="L12" s="16" t="inlineStr">
@@ -2473,7 +2520,7 @@
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>None — needs PRD</t>
+          <t>None — needs PRD (Wave 1)</t>
         </is>
       </c>
       <c r="N12" s="19" t="inlineStr">
@@ -2488,34 +2535,34 @@
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NS-MTH-01, NS-MTH-02</t>
         </is>
       </c>
       <c r="Q12" s="19" t="inlineStr">
         <is>
-          <t>A gap surfaced after the pilot release. No PRD or prototype yet (confidence 0.60) — requirement gathering first, then build. Aligns with the X-dock 'failed condition' work (shared fail-reason + evidence patterns). October so it doesn't compete with the September P0 cluster.</t>
+          <t>High reach × high impact × moderate effort (2.5pw). Split into two waves (Tab 6): Wave 1 ships in September with the P0 cluster (PN-02/PN-03 depend on Cancel/Override landing first); Wave 2 follows in October.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>NS-DA-05</t>
+          <t>4W-NEG</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Driver App</t>
+          <t>Mithril / Driver App</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Local storage + auto-delete (or dedicated logistic app)</t>
+          <t>Negative-scenario handling (failure &amp; exception flows)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Driver phone dies before evidence syncs → billing evidence lost. Local persistence with server-side reconciliation on reconnect. Alternative: a dedicated Dash Logistic app.</t>
+          <t>Model the non-happy paths end-to-end: delivery failed, partial delivery, return-to-origin, exception at gate. Today only the happy path is fully handled.</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
@@ -2525,10 +2572,10 @@
         <v>3</v>
       </c>
       <c r="G13" s="21" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="I13" s="22">
         <f>(E13*F13*G13)/H13</f>
@@ -2544,14 +2591,14 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>Med</t>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Short</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Needs arch decision</t>
+          <t>None — needs PRD</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -2566,19 +2613,19 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>Mobile arch decision (in-app vs new app)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>P1 but scored below Push: 4pw and it needs an architecture call (enhance the shared app vs. spin a dedicated Dash Logistic app). 1-week spike first, then decide. High impact (prevents evidence loss = prevents billing loss) but confidence 0.65 until the arch decision → October.</t>
+          <t>A gap surfaced after the pilot release. No PRD or prototype yet (confidence 0.60) — requirement gathering first, then build. Aligns with the X-dock 'failed condition' work (shared fail-reason + evidence patterns). October so it doesn't compete with the September P0 cluster.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="120" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>NS-DA-02</t>
+          <t>NS-DA-05</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -2588,33 +2635,33 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>EXIM Import/Export tagging (label on trip card)</t>
+          <t>Local storage + auto-delete (or dedicated logistic app)</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>IMPORT / EXPORT badge on Beranda + stepper header — reduces confusion on mixed-lane days.</t>
+          <t>Driver phone dies before evidence syncs → billing evidence lost. Local persistence with server-side reconciliation on reconnect. Alternative: a dedicated Dash Logistic app.</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>0.85</v>
+        <v>0.65</v>
       </c>
       <c r="H14" s="23" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="I14" s="25">
         <f>(E14*F14*G14)/H14</f>
         <v/>
       </c>
-      <c r="J14" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
@@ -2622,14 +2669,14 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="L14" s="9" t="inlineStr">
-        <is>
-          <t>Side</t>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
         </is>
       </c>
       <c r="M14" s="19" t="inlineStr">
         <is>
-          <t>None — needs PRD (dep NS-MTH-03)</t>
+          <t>Needs arch decision</t>
         </is>
       </c>
       <c r="N14" s="19" t="inlineStr">
@@ -2644,19 +2691,19 @@
       </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>NS-MTH-03 (Mithril tag)</t>
+          <t>Mobile arch decision (in-app vs new app)</t>
         </is>
       </c>
       <c r="Q14" s="19" t="inlineStr">
         <is>
-          <t>0.5pw, purely visual. Impact 1 (not 2): drivers rarely mix directions in one day, so it's a clarity win. Piggyback on the Mithril tag rollout in October.</t>
+          <t>P1 but scored below Push: 4pw and it needs an architecture call (enhance the shared app vs. spin a dedicated Dash Logistic app). 1-week spike first, then decide. High impact (prevents evidence loss = prevents billing loss) but confidence 0.65 until the arch decision → October.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="120" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>NS-DA-04</t>
+          <t>NS-DA-02</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -2666,25 +2713,25 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Infinix OS: bypass allow-setting workaround</t>
+          <t>EXIM Import/Export tagging (label on trip card)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Infinix devices block camera/storage permissions by default, preventing Driver App use for a subset of drivers. Vendor-specific fix.</t>
+          <t>IMPORT / EXPORT badge on Beranda + stepper header — reduces confusion on mixed-lane days.</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G15" s="21" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="I15" s="22">
         <f>(E15*F15*G15)/H15</f>
@@ -2707,7 +2754,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>None — needs PRD (dep NS-MTH-03)</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -2722,47 +2769,47 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NS-MTH-03 (Mithril tag)</t>
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>P2 despite high per-user impact — reach is small (only drivers on that OEM). Ship when an Infinix driver is confirmed in the pilot roster, otherwise defer within October.</t>
+          <t>0.5pw, purely visual. Impact 1 (not 2): drivers rarely mix directions in one day, so it's a clarity win. Piggyback on the Mithril tag rollout in October.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="120" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>4W-TRK</t>
+          <t>NS-DA-04</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Mithril / Invoices</t>
+          <t>Driver App</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Tracking invoice 4W</t>
+          <t>Infinix OS: bypass allow-setting workaround</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Import/track 4W invoices by Surat Jalan keyword (4W has no barcode), integrated into the existing Invoices feature.</t>
+          <t>Infinix devices block camera/storage permissions by default, preventing Driver App use for a subset of drivers. Vendor-specific fix.</t>
         </is>
       </c>
       <c r="E16" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" s="24" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="I16" s="25">
         <f>(E16*F16*G16)/H16</f>
@@ -2773,19 +2820,19 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="K16" s="14" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>Med</t>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
         </is>
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>None — post-Sept scope</t>
+          <t>Investigation</t>
         </is>
       </c>
       <c r="N16" s="19" t="inlineStr">
@@ -2800,47 +2847,47 @@
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Invoices feature (existing)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q16" s="19" t="inlineStr">
         <is>
-          <t>Next-phase item from the feature review, scoped after the September rollout so decisions are based on real usage. Connects 4W into the existing Invoices feature; no barcode means it keys off the SJ number.</t>
+          <t>P2 despite high per-user impact — reach is small (only drivers on that OEM). Ship when an Infinix driver is confirmed in the pilot roster, otherwise defer within October.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="120" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>NS-MTH-04</t>
+          <t>4W-TRK</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Mithril / Nexus</t>
+          <t>Mithril / Invoices</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Full sistem UJP — migrate UJP → Mithril (native module)</t>
+          <t>Tracking invoice 4W</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Bring UJP native into Mithril (today it's a separate system in Nexus with an import-only bridge). Removes double-entry, closes the fraud loop, and enables end-to-end finance reporting.</t>
+          <t>Import/track 4W invoices by Surat Jalan keyword (4W has no barcode), integrated into the existing Invoices feature.</t>
         </is>
       </c>
       <c r="E17" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G17" s="21" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I17" s="22">
         <f>(E17*F17*G17)/H17</f>
@@ -2856,14 +2903,14 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr">
-        <is>
-          <t>Side</t>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>None — needs PRD + master-data research</t>
+          <t>None — post-Sept scope</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -2878,47 +2925,47 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>spec control + 'grounds', Basecamp API</t>
+          <t>Invoices feature (existing)</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>Largest scope item (6pw) and the user-flagged 'sistem UJP'. 31 Aug confirmed UJP as the CORE for 4-wheels and prioritized it over P&amp;L (P&amp;L can stay in the existing system for now). UJP lives in Nexus and must integrate with spec control and 'grounds' (which own auto-P&amp;L + control); upload needs master data from several sources → research first. P&amp;L / gross-margin / payroll / 'kois' automation is a later side-quest once all clients use full shipment. Schedule after the pilot is stable.</t>
+          <t>Next-phase item from the feature review, scoped after the September rollout so decisions are based on real usage. Connects 4W into the existing Invoices feature; no barcode means it keys off the SJ number.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="120" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>4W-FLT</t>
+          <t>NS-MTH-04</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Driver App / Fleet</t>
+          <t>Mithril / Nexus</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>Integrasi Fleet — pre-trip QR scan</t>
+          <t>Full sistem UJP — migrate UJP → Mithril (native module)</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Driver scans a vehicle QR at pre-trip so they take the assigned vehicle; the scan result syncs to the Fleet system.</t>
+          <t>Bring UJP native into Mithril (today it's a separate system in Nexus with an import-only bridge). Removes double-entry, closes the fraud loop, and enables end-to-end finance reporting.</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18" s="24" t="n">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="H18" s="23" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="I18" s="25">
         <f>(E18*F18*G18)/H18</f>
@@ -2934,32 +2981,110 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="L18" s="13" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>None — needs PRD + master-data research</t>
+        </is>
+      </c>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>Isumi Karina</t>
+        </is>
+      </c>
+      <c r="O18" s="19" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="P18" s="19" t="inlineStr">
+        <is>
+          <t>spec control + 'grounds', Basecamp API</t>
+        </is>
+      </c>
+      <c r="Q18" s="19" t="inlineStr">
+        <is>
+          <t>Largest scope item (6pw) and the user-flagged 'sistem UJP'. 31 Aug confirmed UJP as the CORE for 4-wheels and prioritized it over P&amp;L (P&amp;L can stay in the existing system for now). UJP lives in Nexus and must integrate with spec control and 'grounds' (which own auto-P&amp;L + control); upload needs master data from several sources → research first. P&amp;L / gross-margin / payroll / 'kois' automation is a later side-quest once all clients use full shipment. Schedule after the pilot is stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>4W-FLT</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Driver App / Fleet</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Integrasi Fleet — pre-trip QR scan</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Driver scans a vehicle QR at pre-trip so they take the assigned vehicle; the scan result syncs to the Fleet system.</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="21" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I19" s="22">
+        <f>(E19*F19*G19)/H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="M18" s="19" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>None — post-Sept scope</t>
         </is>
       </c>
-      <c r="N18" s="19" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Isumi Karina</t>
         </is>
       </c>
-      <c r="O18" s="19" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="P18" s="19" t="inlineStr">
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>Fleet system</t>
         </is>
       </c>
-      <c r="Q18" s="19" t="inlineStr">
+      <c r="Q19" s="4" t="inlineStr">
         <is>
           <t>Cross-system dependency on Fleet. Next-phase, scoped after the September rollout review. Ensures driver-vehicle assignment integrity; lower confidence until the Fleet-side contract is confirmed.</t>
         </is>
@@ -5128,7 +5253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5505,6 +5630,38 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>OQ-11</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>4W EXIM tagging selector — confirm the default workflow mapped to each tag (Export / Import / None) per client, and the 'None' general default.</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>4W</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Ops + Product</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>4W-TAG (tagging selector → default workflow)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Early Sep</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>